<commit_message>
#482: Add manual browser test results (A1, A2, C1-C3, D1-D3)
Covers all remaining P1 cases: location permission flows, Antarctica/
offline/logged-out error handling, and dashboard/phone integration.
Confirms the null-city defect found via the API also reproduces through
real browser GPS and the dashboard-embedded component; found a second
issue where going offline shows Chrome's own error page instead of the
app's documented USA-default fallback.
</commit_message>
<xml_diff>
--- a/data-engineering/tests/Emergency_Contact_Testing_Tracker_482_Somesh-Kennedy.xlsx
+++ b/data-engineering/tests/Emergency_Contact_Testing_Tracker_482_Somesh-Kennedy.xlsx
@@ -2726,52 +2726,418 @@
       </c>
     </row>
     <row r="37">
-      <c r="G37" s="5" t="n"/>
-      <c r="K37" s="5" t="n"/>
-      <c r="L37" s="5" t="n"/>
-      <c r="M37" s="5" t="n"/>
+      <c r="A37" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>United States (real location: Krugerville, TX)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>null (bug) / Lufkin before permission</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Area Detected matches tester's real city/state/country; all 6 numbers match US defaults (911/988)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>Area Detected city shows literal 'null' after granting browser location permission (state/country still correct: Texas, US). Before the permission prompt was answered, an IP-based pre-result correctly showed 'Lufkin, Texas (US)' (acceptable per the test plan, even though the tester's real city is Krugerville).</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>Somesh Kennedy</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>A1 (Allow) - FAIL, Medium defect per section C6 (Area Detected must never show null). Method: reset location permission to Ask, reloaded, clicked Allow. All 6 numbers correct: Police 911, Fire 911, Medical Emergency 911, Ambulance 911, Mental Health Crisis Line 988, Suicide Prevention Hotline 988. Chrome 153.0.8010.48, Windows 11 Home, Lenovo IdeaPad 5, Wi-Fi, no VPN. 2026-10-20.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="G38" s="5" t="n"/>
+      <c r="A38" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Lufkin</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Numbers for the caller's IP country; Area Detected shows the ISP's city (may differ from the tester's real city - that's explicitly OK)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="K38" s="5" t="n"/>
-      <c r="L38" s="5" t="n"/>
-      <c r="M38" s="5" t="n"/>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>Somesh Kennedy</t>
+        </is>
+      </c>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>A2 (Block) - PASS. Method: reset permission, reloaded, clicked Block. Area Detected: Lufkin, Texas (US) - an ISP-based city, differs from the tester's real city (Krugerville), which the test plan explicitly allows. All 6 numbers correct. Chrome 153.0.8010.48, Windows 11 Home, Lenovo IdeaPad 5, Wi-Fi, no VPN. 2026-10-20.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="G39" s="5" t="n"/>
-      <c r="K39" s="5" t="n"/>
-      <c r="L39" s="5" t="n"/>
-      <c r="M39" s="5" t="n"/>
+      <c r="A39" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>N/A (faked via DevTools Sensors)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>AQ</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Antarctica (-75.0, 0.0)</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>No crash; falls back to the caller's IP-country numbers (not 911/988 unless the caller is in the US/Canada)</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>Area Detected city shows literal 'null' (same defect as A1). Numbers correctly fell back to IP-based US defaults since AQ has no dedicated data - that fallback logic is correct.</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>Somesh Kennedy</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>C1 (Antarctica override) - FAIL (same null-city defect as A1, now reproduced via a faked DevTools-Sensors location rather than real GPS - rules out 'specific to real GPS' or 'specific to Antarctica' as the cause). Steps: DevTools -&gt; Sensors panel -&gt; Location: Other, lat=-75.0, lng=0.0, reloaded (DevTools left open). Area Detected: null, Texas (US). All 6 numbers correct per the no-data-location fallback. No console errors observed. Chrome 153.0.8010.48, Windows 11 Home, Lenovo IdeaPad 5, Wi-Fi, no VPN. 2026-10-20.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="G40" s="5" t="n"/>
+      <c r="A40" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Record what happens; known issue says logged-out visitors may see US 911/988</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="K40" s="5" t="n"/>
-      <c r="L40" s="5" t="n"/>
-      <c r="M40" s="5" t="n"/>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>Somesh Kennedy</t>
+        </is>
+      </c>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>C2 (logged-out visitor) - Observation, not a fail. Logged out, then opened /emergency-contact directly. Page rendered briefly (~1s) then automatically redirected to the login page; no error message shown; no emergency numbers were ever displayed to the logged-out visitor. This differs from (and looks safer than) the documented known issue, which describes logged-out visitors possibly being shown incorrect US defaults rather than being redirected to login. Chrome 153.0.8010.48, Windows 11 Home, Lenovo IdeaPad 5, Wi-Fi, no VPN. 2026-10-20.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="G41" s="5" t="n"/>
-      <c r="K41" s="5" t="n"/>
-      <c r="L41" s="5" t="n"/>
-      <c r="M41" s="5" t="n"/>
+      <c r="A41" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>No crash or blank page; expect 'Using default emergency numbers - USA' (known issue, record it)</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>Chrome's native ERR_INTERNET_DISCONNECTED page shown instead of the app; no part of the Saayam UI rendered at all, not even a fallback.</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>Somesh Kennedy</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>C3 (offline) - FAIL, discrepancy from the documented expectation. Steps: loaded the page once normally, DevTools -&gt; Network tab, changed throttling from 'No throttling' to 'Offline', reloaded. Result: a full browser-level connection failure (Chrome's own ERR_INTERNET_DISCONNECTED interstitial), not the app's documented 'USA defaults' fallback UI. Suggests no service worker / offline app-shell caching - a hard reload while offline can't render any part of the page. Different from, and arguably worse than, what the issue describes as the known issue, since nothing of the app loads at all. Throttling was reset to 'No throttling' afterward. Chrome 153.0.8010.48, Windows 11 Home, Lenovo IdeaPad 5, Wi-Fi, no VPN. 2026-10-20.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="G42" s="5" t="n"/>
-      <c r="K42" s="5" t="n"/>
-      <c r="L42" s="5" t="n"/>
-      <c r="M42" s="5" t="n"/>
+      <c r="A42" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>United States (real location: Krugerville, TX)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>null (bug)</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Same numbers and Area Detected as the standalone page (A1)</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>Same null-city defect as A1 reproduces here too.</t>
+        </is>
+      </c>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>Somesh Kennedy</t>
+        </is>
+      </c>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>D1 (dashboard -&gt; Emergency Contact button) - PASS on its own criterion (consistent with A1), but carries forward A1's null-city defect. Steps: Super Admin Dashboard -&gt; All Requests -&gt; opened a Request ID -&gt; clicked the Emergency Contact button -&gt; clicked Allow on the location prompt. Area Detected: null, Texas (US). All 6 numbers correct. Confirms the dashboard-embedded button uses the same shared component as the standalone page (same bug, same output). Chrome 153.0.8010.48, Windows 11 Home, Lenovo IdeaPad 5, Wi-Fi, no VPN. 2026-10-20.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="G43" s="5" t="n"/>
+      <c r="A43" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>Returns to the dashboard</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="K43" s="5" t="n"/>
-      <c r="L43" s="5" t="n"/>
-      <c r="M43" s="5" t="n"/>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>Somesh Kennedy</t>
+        </is>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>D2 (back to dashboard) - PASS. Clicked 'Back to Dashboard' from the Emergency Contact view opened via D1; correctly returned to the dashboard. Chrome 153.0.8010.48, Windows 11 Home, Lenovo IdeaPad 5, Wi-Fi, no VPN. 2026-10-20.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="G44" s="5" t="n"/>
+      <c r="A44" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>N/A (phone test)</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>The phone dialer opens with exactly that number</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="K44" s="5" t="n"/>
-      <c r="L44" s="5" t="n"/>
-      <c r="M44" s="5" t="n"/>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>Somesh Kennedy</t>
+        </is>
+      </c>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>D3 (phone dialer) - PASS. On a phone, opened the standalone page, allowed location, tapped the Fire Department row. The OS presented an app chooser since multiple apps are registered for tel: links (expected OS behavior, not a bug) - selected the Phone/Dialer app, which opened with the number pre-filled, exactly matching what the page showed. Did not press call. (Phone model/OS version not recorded for this test.) 2026-10-20.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="G45" s="5" t="n"/>

</xml_diff>